<commit_message>
style(output): readability polish (fonts, spacing, tables, xlsx widths) with zero text changes; CA Soalan JPK PDFs re-exported
104 generated docx + 14 JPK-format Soalan polished per _tools/READABILITY-SPEC.md (Arial 11, 1.15 spacing, bold section labels, Table Grid with shaded headers); before/after text dumps identical for every file. 5 xlsx: header styling, wrap, widths, freeze panes; values and formulas unchanged (Lampiran 5 still 6 sheets / 2,523 formulas). Buku Teks PDFs regenerated (164 pp CU book, 347 pp CA book). Soalan JPK: MENGANDUNGI page counts re-patched (6/5) and PDFs re-exported. Added _tools/Export-Pdf.ps1 (one Word process per file — robust against COM RPC drops).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/video-film-editing/output/02 4.2 Penjajaran Jam Latihan CA-CU/4.2_Penjajaran Jam Latihan CA_CU_EU Program ADI Pekerjaan (IT-072).xlsx
+++ b/video-film-editing/output/02 4.2 Penjajaran Jam Latihan CA-CU/4.2_Penjajaran Jam Latihan CA_CU_EU Program ADI Pekerjaan (IT-072).xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-30340" yWindow="2240" windowWidth="21820" windowHeight="13900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PENJAJARAN CU" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="PENJAJARAN CU" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'PENJAJARAN CU'!$A$1:$E$22</definedName>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Aptos Narrow"/>
       <color theme="1"/>
@@ -91,8 +91,11 @@
       <color theme="1"/>
       <sz val="14"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -151,6 +154,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -290,7 +299,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -379,6 +388,84 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -660,28 +747,29 @@
   <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="24.6640625" customWidth="1" style="24" min="1" max="1"/>
-    <col width="38.33203125" customWidth="1" style="24" min="2" max="2"/>
-    <col width="20.5" customWidth="1" style="24" min="3" max="3"/>
-    <col width="26.6640625" customWidth="1" style="24" min="4" max="4"/>
-    <col width="18.6640625" customWidth="1" style="24" min="5" max="5"/>
+    <col width="60" customWidth="1" style="24" min="1" max="1"/>
+    <col width="60" customWidth="1" style="24" min="2" max="2"/>
+    <col width="33" customWidth="1" style="24" min="3" max="3"/>
+    <col width="50" customWidth="1" style="24" min="4" max="4"/>
+    <col width="28" customWidth="1" style="24" min="5" max="5"/>
     <col width="8.6640625" customWidth="1" style="24" min="6" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1" s="24">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">PENJAJARAN JAM LATIHAN KOMPETENSI UNIT (CU) MENGIKUT ADi BAGI HOURS </t>
         </is>
       </c>
+      <c r="E1" s="35" t="n"/>
     </row>
     <row r="2" ht="14.25" customHeight="1" s="24">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="36" t="inlineStr">
         <is>
           <t>SEKTOR</t>
         </is>
       </c>
-      <c r="B2" s="20" t="inlineStr">
+      <c r="B2" s="37" t="inlineStr">
         <is>
           <t>INFORMATION TECHNOLOGY &amp; COMMUNICATION (ICT)</t>
         </is>
@@ -691,12 +779,12 @@
       <c r="E2" s="33" t="n"/>
     </row>
     <row r="3" ht="14.25" customHeight="1" s="24">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="36" t="inlineStr">
         <is>
           <t>SUB-SEKTOR</t>
         </is>
       </c>
-      <c r="B3" s="20" t="inlineStr">
+      <c r="B3" s="37" t="inlineStr">
         <is>
           <t>DIGITAL CREATIVE</t>
         </is>
@@ -706,12 +794,12 @@
       <c r="E3" s="33" t="n"/>
     </row>
     <row r="4" ht="14.25" customHeight="1" s="24">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="36" t="inlineStr">
         <is>
           <t>KOD / NOSS</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="38" t="inlineStr">
         <is>
           <t>IT-072-3:2012 VIDEO / FILM (EDITING)</t>
         </is>
@@ -721,12 +809,12 @@
       <c r="E4" s="33" t="n"/>
     </row>
     <row r="5" ht="14.25" customHeight="1" s="24">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="36" t="inlineStr">
         <is>
           <t>TAHAP</t>
         </is>
       </c>
-      <c r="B5" s="20" t="n">
+      <c r="B5" s="37" t="n">
         <v>3</v>
       </c>
       <c r="C5" s="33" t="n"/>
@@ -734,12 +822,12 @@
       <c r="E5" s="33" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1" s="24">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="36" t="inlineStr">
         <is>
           <t>Jenis Program</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="37" t="inlineStr">
         <is>
           <t>Mengikut Tahap (NOSS Bermula Tahap 3)</t>
         </is>
@@ -749,284 +837,345 @@
       <c r="E6" s="33" t="n"/>
     </row>
     <row r="7" ht="14.25" customHeight="1" s="24">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="36" t="inlineStr">
         <is>
           <t>Jumlah Jam Latihan ADI</t>
         </is>
       </c>
-      <c r="B7" s="20" t="n">
+      <c r="B7" s="37" t="n">
         <v>2880</v>
       </c>
-      <c r="C7" s="12" t="n"/>
-      <c r="D7" s="12" t="n"/>
-      <c r="E7" s="12" t="n"/>
+      <c r="C7" s="39" t="n"/>
+      <c r="D7" s="39" t="n"/>
+      <c r="E7" s="39" t="n"/>
     </row>
     <row r="8" ht="14.25" customHeight="1" s="24">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="36" t="inlineStr">
         <is>
           <t>Jumlah Jam Latihan Teori</t>
         </is>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="37" t="n">
         <v>576</v>
       </c>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="12" t="n"/>
-      <c r="E8" s="12" t="n"/>
+      <c r="C8" s="39" t="n"/>
+      <c r="D8" s="39" t="n"/>
+      <c r="E8" s="39" t="n"/>
     </row>
     <row r="9" ht="48" customHeight="1" s="24">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="40" t="inlineStr">
         <is>
           <t>KOD CU</t>
         </is>
       </c>
-      <c r="B9" s="29" t="inlineStr">
+      <c r="B9" s="41" t="inlineStr">
         <is>
           <t>TITLE COMPETENCY UNIT (CU)</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="40" t="inlineStr">
         <is>
           <t>JAM LATIHAN CA/CU/EU (ADi)</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="40" t="inlineStr">
         <is>
           <t>Jumlah Hari Teori 
 (Jam CA/CU/EU ÷ 8 Jam sehari)</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="40" t="inlineStr">
         <is>
           <t>Pundaran Jumlah Hari Teori</t>
         </is>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1" s="24">
-      <c r="A10" s="26" t="inlineStr">
+      <c r="A10" s="42" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="B10" s="31" t="inlineStr">
+      <c r="B10" s="43" t="inlineStr">
         <is>
           <t>Core Abilities Tahap 1, 2 &amp; 3</t>
         </is>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="44" t="n">
         <v>80</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="45" t="n">
         <v>10</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="46" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1" s="24">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="47" t="inlineStr">
         <is>
           <t>C01</t>
         </is>
       </c>
-      <c r="B11" s="32" t="inlineStr">
+      <c r="B11" s="48" t="inlineStr">
         <is>
           <t>Visual Editing Project Analysis</t>
         </is>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="49">
         <f>($B$8-$C$10)/ROWS($A$11:$A$15)</f>
         <v/>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="50">
         <f>C11/8</f>
         <v/>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="51" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1" s="24">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="47" t="inlineStr">
         <is>
           <t>C02</t>
         </is>
       </c>
-      <c r="B12" s="32" t="inlineStr">
+      <c r="B12" s="48" t="inlineStr">
         <is>
           <t>Visual Editing Preparation</t>
         </is>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="49">
         <f>($B$8-$C$10)/ROWS($A$11:$A$15)</f>
         <v/>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="50">
         <f>C12/8</f>
         <v/>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="51" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1" s="24">
-      <c r="A13" s="27" t="inlineStr">
+      <c r="A13" s="47" t="inlineStr">
         <is>
           <t>C03</t>
         </is>
       </c>
-      <c r="B13" s="32" t="inlineStr">
+      <c r="B13" s="48" t="inlineStr">
         <is>
           <t>Offline Visual Editing</t>
         </is>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="49">
         <f>($B$8-$C$10)/ROWS($A$11:$A$15)</f>
         <v/>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="50">
         <f>C13/8</f>
         <v/>
       </c>
-      <c r="E13" s="17" t="n">
+      <c r="E13" s="51" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1" s="24">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="47" t="inlineStr">
         <is>
           <t>C04</t>
         </is>
       </c>
-      <c r="B14" s="32" t="inlineStr">
+      <c r="B14" s="48" t="inlineStr">
         <is>
           <t>Audio Sweetening</t>
         </is>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="49">
         <f>($B$8-$C$10)/ROWS($A$11:$A$15)</f>
         <v/>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="50">
         <f>C14/8</f>
         <v/>
       </c>
-      <c r="E14" s="17" t="n">
+      <c r="E14" s="51" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1" s="24">
-      <c r="A15" s="27" t="inlineStr">
+      <c r="A15" s="47" t="inlineStr">
         <is>
           <t>C05</t>
         </is>
       </c>
-      <c r="B15" s="32" t="inlineStr">
+      <c r="B15" s="48" t="inlineStr">
         <is>
           <t>Online Visual Editing</t>
         </is>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="49">
         <f>($B$8-$C$10)/ROWS($A$11:$A$15)</f>
         <v/>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="50">
         <f>C15/8</f>
         <v/>
       </c>
-      <c r="E15" s="17" t="n">
+      <c r="E15" s="51" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1" s="24" thickBot="1">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="52" t="inlineStr">
         <is>
           <t>JUMLAH</t>
         </is>
       </c>
-      <c r="B16" s="33" t="n"/>
-      <c r="C16" s="8" t="n">
+      <c r="B16" s="53" t="n"/>
+      <c r="C16" s="54" t="n">
         <v>576</v>
       </c>
-      <c r="D16" s="22">
+      <c r="D16" s="52">
         <f>SUM(D11:D15)</f>
         <v/>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="55">
         <f>SUM(E11:E15)</f>
         <v/>
       </c>
     </row>
-    <row r="17" ht="14.25" customHeight="1" s="24" thickBot="1" thickTop="1"/>
+    <row r="17" ht="14.25" customHeight="1" s="24" thickBot="1" thickTop="1">
+      <c r="A17" s="35" t="n"/>
+      <c r="C17" s="35" t="n"/>
+      <c r="D17" s="35" t="n"/>
+      <c r="E17" s="35" t="n"/>
+    </row>
     <row r="18" ht="14.25" customHeight="1" s="24" thickTop="1">
-      <c r="B18" s="1" t="inlineStr">
+      <c r="A18" s="35" t="n"/>
+      <c r="B18" s="56" t="inlineStr">
         <is>
           <t>RK = RELATED KNOWLEDGE / THEORY</t>
         </is>
       </c>
-      <c r="C18" s="19" t="n"/>
+      <c r="C18" s="57" t="n"/>
+      <c r="D18" s="35" t="n"/>
+      <c r="E18" s="35" t="n"/>
     </row>
     <row r="19" ht="14.25" customHeight="1" s="24">
-      <c r="B19" s="1" t="inlineStr">
+      <c r="A19" s="35" t="n"/>
+      <c r="B19" s="56" t="inlineStr">
         <is>
           <t>RS = RELATED SKILL / PRACTICAL</t>
         </is>
       </c>
+      <c r="C19" s="35" t="n"/>
     </row>
     <row r="20" ht="14.25" customHeight="1" s="24">
-      <c r="B20" s="1" t="n"/>
+      <c r="A20" s="35" t="n"/>
+      <c r="B20" s="56" t="n"/>
     </row>
     <row r="21" ht="14.25" customHeight="1" s="24">
-      <c r="B21" s="1" t="n"/>
+      <c r="A21" s="35" t="n"/>
+      <c r="B21" s="56" t="n"/>
     </row>
     <row r="22" ht="14.25" customHeight="1" s="24">
-      <c r="B22" s="1" t="n"/>
-    </row>
-    <row r="23" ht="14.25" customHeight="1" s="24"/>
+      <c r="A22" s="35" t="n"/>
+      <c r="B22" s="56" t="n"/>
+    </row>
+    <row r="23" ht="14.25" customHeight="1" s="24">
+      <c r="A23" s="35" t="n"/>
+      <c r="B23" s="35" t="n"/>
+      <c r="C23" s="35" t="n"/>
+      <c r="D23" s="35" t="n"/>
+      <c r="E23" s="35" t="n"/>
+    </row>
     <row r="24" ht="14.25" customHeight="1" s="24">
-      <c r="B24" s="2" t="inlineStr">
+      <c r="A24" s="35" t="n"/>
+      <c r="B24" s="58" t="inlineStr">
         <is>
           <t>1 Hari 8 Jam</t>
         </is>
       </c>
+      <c r="C24" s="35" t="n"/>
+      <c r="D24" s="35" t="n"/>
+      <c r="E24" s="35" t="n"/>
     </row>
     <row r="25" ht="14.25" customHeight="1" s="24">
-      <c r="B25" s="2" t="inlineStr">
+      <c r="A25" s="35" t="n"/>
+      <c r="B25" s="58" t="inlineStr">
         <is>
           <t xml:space="preserve">1Minggu 5 Hari = 5 x 8 Jam = 40 Jam </t>
         </is>
       </c>
+      <c r="C25" s="35" t="n"/>
+      <c r="D25" s="35" t="n"/>
+      <c r="E25" s="35" t="n"/>
     </row>
     <row r="26" ht="14.25" customHeight="1" s="24">
-      <c r="B26" s="2" t="inlineStr">
+      <c r="A26" s="35" t="n"/>
+      <c r="B26" s="58" t="inlineStr">
         <is>
           <t>1 bulan x 4 Minggu = 4 x 40 jam = 160 Jam</t>
         </is>
       </c>
-    </row>
-    <row r="27" ht="14.25" customHeight="1" s="24"/>
+      <c r="C26" s="35" t="n"/>
+      <c r="D26" s="35" t="n"/>
+      <c r="E26" s="35" t="n"/>
+    </row>
+    <row r="27" ht="14.25" customHeight="1" s="24">
+      <c r="A27" s="35" t="n"/>
+      <c r="B27" s="35" t="n"/>
+      <c r="C27" s="35" t="n"/>
+      <c r="D27" s="35" t="n"/>
+      <c r="E27" s="35" t="n"/>
+    </row>
     <row r="28" ht="14.25" customHeight="1" s="24">
-      <c r="B28" s="2" t="inlineStr">
+      <c r="A28" s="35" t="n"/>
+      <c r="B28" s="58" t="inlineStr">
         <is>
           <t>1 bulan = 160 jam</t>
         </is>
       </c>
-    </row>
-    <row r="29" ht="14.25" customHeight="1" s="24"/>
+      <c r="C28" s="35" t="n"/>
+      <c r="D28" s="35" t="n"/>
+      <c r="E28" s="35" t="n"/>
+    </row>
+    <row r="29" ht="14.25" customHeight="1" s="24">
+      <c r="A29" s="35" t="n"/>
+      <c r="B29" s="35" t="n"/>
+      <c r="C29" s="35" t="n"/>
+      <c r="D29" s="35" t="n"/>
+      <c r="E29" s="35" t="n"/>
+    </row>
     <row r="30" ht="14.25" customHeight="1" s="24">
-      <c r="B30" s="2" t="inlineStr">
+      <c r="A30" s="35" t="n"/>
+      <c r="B30" s="58" t="inlineStr">
         <is>
           <t>18 bulan x 160 jam = 2880 Jam</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="14.25" customHeight="1" s="24"/>
+      <c r="C30" s="35" t="n"/>
+      <c r="D30" s="35" t="n"/>
+      <c r="E30" s="35" t="n"/>
+    </row>
+    <row r="31" ht="14.25" customHeight="1" s="24">
+      <c r="A31" s="35" t="n"/>
+      <c r="B31" s="35" t="n"/>
+      <c r="C31" s="35" t="n"/>
+      <c r="D31" s="35" t="n"/>
+      <c r="E31" s="35" t="n"/>
+    </row>
     <row r="32" ht="14.25" customHeight="1" s="24">
-      <c r="B32" s="3" t="inlineStr">
+      <c r="A32" s="35" t="n"/>
+      <c r="B32" s="59" t="inlineStr">
         <is>
           <t>Jumlah Jam Pengetahuan (20%) untuk kiraan CA/CU/EU = (2880 x 20%) = 576 Jam</t>
         </is>
       </c>
+      <c r="C32" s="35" t="n"/>
+      <c r="D32" s="35" t="n"/>
+      <c r="E32" s="35" t="n"/>
     </row>
     <row r="33" ht="14.25" customHeight="1" s="24"/>
     <row r="34" ht="14.25" customHeight="1" s="24"/>

</xml_diff>